<commit_message>
Bear case re-runs in progress (evidence audit)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/KO/2026-10-13/bear/scratch/base_check/dcf.xlsx
+++ b/runs/KO/2026-10-13/bear/scratch/base_check/dcf.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -580,7 +580,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Risk-free rate (US 10y)</t>
+          <t>Risk-free rate (10-year government bond in USD, the cash-flow currency)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.05</v>
+        <v>0.042</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -715,161 +715,191 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net debt (USD m)</t>
+          <t>Share buybacks after the balance sheet date (USD m)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>29686</v>
+        <v>0</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) balance sheet at 31 Dec 2025: loans and notes payable 1,551 + current maturities of LTD 1,822 + LTD 42,119 - cash 10,270 - short-term investments 3,602 - marketable securities 1,934. No finance-lease liability is disclosed separately (none inside or outside). EXCLUDES CCBA debt 1,435 and cash 178 (in held-for-sale).</t>
+          <t>not in this brief's bridge (0)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lease liabilities not in net debt (USD m)</t>
+          <t>Bridge items already priced at the valuation date, not grown (USD m)</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1722</v>
+        <v>39539.5</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 10: total operating lease liabilities 1,722 (current 321 in payables, noncurrent 1,401 in other noncurrent liabilities); NOT in net debt, so deducted separately.</t>
+          <t>Listed equity stakes at run-date (13 Oct 2026) market value, the 39,539.5 inside 'associates' (data/associates_rollforward_check.csv, Yahoo/FRED). Added by the evidence audit 15 Oct 2026: KO was valued before the desk learned to keep run-date values out of the roll-forward (mistakes log row 24)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Minority interests at book (USD m)</t>
+          <t>Net debt (USD m)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>2106</v>
+        <v>29686</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) balance sheet: equity attributable to noncontrolling interests 2,106 (book; includes the 40% India bottling NCI sold July 2025 and the outside shareholders of CCBA - see FLAG) FLAG (PM informed 2026-10-13): includes CCBA's outside shareholder (Gutsche 33.5%), not disclosed; full amount deducted (conservative, up to c.USD 1.1bn too much).</t>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) balance sheet at 31 Dec 2025: loans and notes payable 1,551 + current maturities of LTD 1,822 + LTD 42,119 - cash 10,270 - short-term investments 3,602 - marketable securities 1,934. No finance-lease liability is disclosed separately (none inside or outside). EXCLUDES CCBA debt 1,435 and cash 178 (in held-for-sale).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Minorities' share of operating profit (proportionate method; blank = use book)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
+          <t>Lease liabilities not in net debt (USD m)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>1722</v>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PM assumption (briefs/KO.yaml)</t>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 10: total operating lease liabilities 1,722 (current 321 in payables, noncurrent 1,401 in other noncurrent liabilities); NOT in net debt, so deducted separately.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pension deficit (USD m)</t>
+          <t>Minority interests at book (USD m)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0</v>
+        <v>2106</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 14: pension plans net ASSET 295, other postretirement net liability 112 = net surplus 183; brief rule 0 if in surplus. Gross accrued liability of deficit plans 863 (MD&amp;A) - see notes.</t>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) balance sheet: equity attributable to noncontrolling interests 2,106 (book; includes the 40% India bottling NCI sold July 2025 and the outside shareholders of CCBA - see FLAG) FLAG (PM informed 2026-10-13): includes CCBA's outside shareholder (Gutsche 33.5%), not disclosed; full amount deducted (conservative, up to c.USD 1.1bn too much).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Associates and equity stakes (USD m)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>46625.5</v>
-      </c>
+          <t>Minorities' share of operating profit (proportionate method; blank = use book)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Listed stakes at run-date market value 39539.5 (data/associates_rollforward_check.csv: 31 Dec 2025 fair values from FY25 10-K x price and FX change to 13 Oct 2026, Yahoo/FRED) + unlisted equity-method investments at book 6,236 (FY25 10-K: 20,235 - listed book 13,999) + retained 25% of CCBA at deal value 850 (0.25 x USD 3.4bn, Coca-Cola HBC CCBA acquisition announcement, 21 Oct 2025 (factsheet https://www.coca-colahellenic.com/content/dam/cch/us/documents/investors-and-financial/2026-q1-trading-update/coca-cola-hbc-factsheet-ccba-acquisition-q1-2026.pdf.downloadasset.pdf and acquisition presentation): CCBA 2024 net sales revenue EUR 3,357m, EBIT EUR 246m; KO sells 41.5% for USD 1.3bn, keeps 25%; 100% equity value USD 3.4bn. Seen via web search; page not reachable from this environment, PM asked to verify). PM rule: listed stakes at run-date market value</t>
+          <t>PM assumption (briefs/KO.yaml)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Disposal proceeds not in net debt (USD m)</t>
+          <t>Pension deficit (USD m)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KO's 41.5% of CCBA sold for USD 1.3bn, not yet received (Q2 2026 10-Q: not closed). Coca-Cola HBC CCBA acquisition announcement, 21 Oct 2025 (factsheet https://www.coca-colahellenic.com/content/dam/cch/us/documents/investors-and-financial/2026-q1-trading-update/coca-cola-hbc-factsheet-ccba-acquisition-q1-2026.pdf.downloadasset.pdf and acquisition presentation): CCBA 2024 net sales revenue EUR 3,357m, EBIT EUR 246m; KO sells 41.5% for USD 1.3bn, keeps 25%; 100% equity value USD 3.4bn. Seen via web search; page not reachable from this environment, PM asked to verify. PM decision 2026-10-13</t>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 14: pension plans net ASSET 295, other postretirement net liability 112 = net surplus 183; brief rule 0 if in surplus. Gross accrued liability of deficit plans 863 (MD&amp;A) - see notes.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Restructuring cash still to pay (USD m)</t>
+          <t>Associates and equity stakes (USD m)</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0</v>
+        <v>46625.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 19: productivity and reinvestment program (2012-2017) 'substantially completed' at 31 Dec 2025 (FY25 charge 97); no new programme announced in the Q1/Q2 2026 10-Qs.</t>
+          <t>Listed stakes at run-date market value 39539.5 (data/associates_rollforward_check.csv: 31 Dec 2025 fair values from FY25 10-K x price and FX change to 13 Oct 2026, Yahoo/FRED) + unlisted equity-method investments at book 6,236 (FY25 10-K: 20,235 - listed book 13,999) + retained 25% of CCBA at deal value 850 (0.25 x USD 3.4bn, Coca-Cola HBC CCBA acquisition announcement, 21 Oct 2025 (factsheet https://www.coca-colahellenic.com/content/dam/cch/us/documents/investors-and-financial/2026-q1-trading-update/coca-cola-hbc-factsheet-ccba-acquisition-q1-2026.pdf.downloadasset.pdf and acquisition presentation): CCBA 2024 net sales revenue EUR 3,357m, EBIT EUR 246m; KO sells 41.5% for USD 1.3bn, keeps 25%; 100% equity value USD 3.4bn. Seen via web search; page not reachable from this environment, PM asked to verify). PM rule: listed stakes at run-date market value</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Contingent liabilities assumed paid, e.g. a lost tax case (USD m)</t>
+          <t>Disposal proceeds not in net debt (USD m)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>14000</v>
+        <v>1300</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Potential IRS tax and interest 2010-2025 at 31 Dec 2025, KO FY25 10-K (accession 0001628280-26-010047; XBRL ko:IncrementalTaxAndInterestLiability = 14,000m). PM decision 2026-10-13: assume KO loses; H1 2026 accrual (USD 900m, Q2 2026 10-Q) excluded because the 23.7% tax rate already charges 2026 onwards (mistakes log row 17)</t>
+          <t>KO's 41.5% of CCBA sold for USD 1.3bn, not yet received (Q2 2026 10-Q: not closed). Coca-Cola HBC CCBA acquisition announcement, 21 Oct 2025 (factsheet https://www.coca-colahellenic.com/content/dam/cch/us/documents/investors-and-financial/2026-q1-trading-update/coca-cola-hbc-factsheet-ccba-acquisition-q1-2026.pdf.downloadasset.pdf and acquisition presentation): CCBA 2024 net sales revenue EUR 3,357m, EBIT EUR 246m; KO sells 41.5% for USD 1.3bn, keeps 25%; 100% equity value USD 3.4bn. Seen via web search; page not reachable from this environment, PM asked to verify. PM decision 2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ordinary shares (m)</t>
+          <t>Restructuring cash still to pay (USD m)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>4302</v>
+        <v>0</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) XBRL: 7,040m issued (us-gaap:CommonStockSharesIssued) - 2,738m treasury (us-gaap:TreasuryStockCommonShares) at 31 Dec 2025. Check: Q2 2026 10-Q cover 4,302,549,243 at 27 Jul 2026.</t>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) Note 19: productivity and reinvestment program (2012-2017) 'substantially completed' at 31 Dec 2025 (FY25 charge 97); no new programme announced in the Q1/Q2 2026 10-Qs.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Contingent liabilities assumed paid, e.g. a lost tax case (USD m)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Potential IRS tax and interest 2010-2025 at 31 Dec 2025, KO FY25 10-K (accession 0001628280-26-010047; XBRL ko:IncrementalTaxAndInterestLiability = 14,000m). PM decision 2026-10-13: assume KO loses; H1 2026 accrual (USD 900m, Q2 2026 10-Q) excluded because the 23.7% tax rate already charges 2026 onwards (mistakes log row 17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ordinary shares (m)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>4302</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KO FY25 10-K (accession 0001628280-26-010047, filed 2026-02-20, https://www.sec.gov/Archives/edgar/data/21344/000162828026010047/ko-20251231.htm) XBRL: 7,040m issued (us-gaap:CommonStockSharesIssued) - 2,738m treasury (us-gaap:TreasuryStockCommonShares) at 31 Dec 2025. Check: Q2 2026 10-Q cover 4,302,549,243 at 27 Jul 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Share price (USD)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>90.12000274658203</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Yahoo Finance KO close (US dollars), 2026-10-13</t>
         </is>
@@ -1321,7 +1351,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>8936.606437882856</v>
+        <v>9107.107949281915</v>
       </c>
     </row>
     <row r="16">
@@ -1347,7 +1377,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.08265499999999999</v>
+        <v>0.0777822</v>
       </c>
     </row>
     <row r="18">
@@ -1375,7 +1405,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.07998361189599999</v>
+        <v>0.075457365432</v>
       </c>
     </row>
     <row r="20">
@@ -1389,7 +1419,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>49362.739673712</v>
+        <v>49863.77626134607</v>
       </c>
     </row>
     <row r="21">
@@ -1417,7 +1447,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>210781.4805365465</v>
+        <v>227984.7667641451</v>
       </c>
     </row>
     <row r="23">
@@ -1431,7 +1461,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>149092.297240781</v>
+        <v>164337.4098355939</v>
       </c>
     </row>
     <row r="24">
@@ -1445,7 +1475,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>198455.036914493</v>
+        <v>214201.18609694</v>
       </c>
     </row>
     <row r="25">
@@ -1455,7 +1485,7 @@
         </is>
       </c>
       <c r="B25" s="4">
-        <f>IF(ISBLANK(Inputs!$B$22),Inputs!$B$21,Inputs!$B$22*B24)</f>
+        <f>IF(ISBLANK(Inputs!$B$24),Inputs!$B$23,Inputs!$B$24*B24)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="n">
@@ -1469,11 +1499,11 @@
         </is>
       </c>
       <c r="B26" s="4">
-        <f>B24-Inputs!$B$19-Inputs!$B$20-B25-Inputs!$B$23-Inputs!$B$26-Inputs!$B$27+Inputs!$B$24+Inputs!$B$25</f>
+        <f>B24-Inputs!$B$21-Inputs!$B$22-B25-Inputs!$B$25-Inputs!$B$28-Inputs!$B$29+Inputs!$B$26+Inputs!$B$27</f>
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>198866.536914493</v>
+        <v>214612.68609694</v>
       </c>
     </row>
     <row r="27">
@@ -1483,11 +1513,11 @@
         </is>
       </c>
       <c r="B27" s="4">
-        <f>B26*(1+B17)^Inputs!$B$17-Inputs!$B$18</f>
+        <f>(B26-Inputs!$B$20)*(1+B17)^Inputs!$B$17+Inputs!$B$20-Inputs!$B$18-Inputs!$B$19</f>
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>204794.4443411516</v>
+        <v>218355.5743686419</v>
       </c>
     </row>
     <row r="28">
@@ -1497,11 +1527,11 @@
         </is>
       </c>
       <c r="B28" s="4">
-        <f>B27/Inputs!$B$28</f>
+        <f>B27/Inputs!$B$30</f>
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>47.60447334754803</v>
+        <v>50.75675833766664</v>
       </c>
     </row>
     <row r="29">
@@ -1511,11 +1541,11 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>B28/Inputs!$B$29-1</f>
+        <f>B28/Inputs!$B$31-1</f>
         <v/>
       </c>
       <c r="C29" s="6" t="n">
-        <v>-0.4717657357</v>
+        <v>-0.4367869863</v>
       </c>
     </row>
   </sheetData>

</xml_diff>